<commit_message>
Update datasets, figures, and add new scripts
Updated multiple CSV and Excel datasets, modified statistical figures and calculation scripts, and added new presentation and utility files. Replaced and renamed mutation output CSV, added a new PowerPoint presentation, and introduced a new Python script for LLM checks.
</commit_message>
<xml_diff>
--- a/stat/data.xlsx
+++ b/stat/data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\test\stat\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB53D1D1-9FBB-450D-84BD-EA7024D1EAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB5BED9-3025-4034-8716-D4AD39290DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="14">
   <si>
     <t>gpt-4o</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -76,6 +76,10 @@
   </si>
   <si>
     <t>overcorrection</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>pass@6</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -401,10 +405,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>2</v>
       </c>
@@ -420,13 +424,31 @@
       <c r="F1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="H1" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" t="s">
+        <v>8</v>
+      </c>
+      <c r="M1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -445,8 +467,23 @@
       <c r="F3">
         <v>1.5811999999999999</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="H3">
+        <v>38</v>
+      </c>
+      <c r="I3">
+        <v>26.53</v>
+      </c>
+      <c r="J3">
+        <v>3.92</v>
+      </c>
+      <c r="K3">
+        <v>101.73</v>
+      </c>
+      <c r="L3">
+        <v>1.4113</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -466,27 +503,27 @@
         <v>13.4636</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -505,8 +542,23 @@
       <c r="F9">
         <v>17.4329</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="H9">
+        <v>43</v>
+      </c>
+      <c r="I9">
+        <v>20.41</v>
+      </c>
+      <c r="J9">
+        <v>7.84</v>
+      </c>
+      <c r="K9">
+        <v>2633.25</v>
+      </c>
+      <c r="L9">
+        <v>30.0015</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -526,12 +578,12 @@
         <v>155.00290000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -550,8 +602,23 @@
       <c r="F12">
         <v>34.570399999999999</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="H12">
+        <v>38</v>
+      </c>
+      <c r="I12">
+        <v>30.61</v>
+      </c>
+      <c r="J12">
+        <v>7.84</v>
+      </c>
+      <c r="K12">
+        <v>4222.12</v>
+      </c>
+      <c r="L12">
+        <v>42.000700000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>1</v>
       </c>
@@ -571,12 +638,12 @@
         <v>78.007099999999994</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -595,8 +662,23 @@
       <c r="F15">
         <v>1.4267000000000001</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="H15">
+        <v>16</v>
+      </c>
+      <c r="I15">
+        <v>69.39</v>
+      </c>
+      <c r="J15">
+        <v>1.96</v>
+      </c>
+      <c r="K15">
+        <v>197.15</v>
+      </c>
+      <c r="L15">
+        <v>1.8134999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>1</v>
       </c>
@@ -616,12 +698,12 @@
         <v>27.958100000000002</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -640,8 +722,26 @@
       <c r="F18">
         <v>17.093699999999998</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="H18">
+        <v>17</v>
+      </c>
+      <c r="I18">
+        <v>67.349999999999994</v>
+      </c>
+      <c r="J18">
+        <v>1.96</v>
+      </c>
+      <c r="K18">
+        <v>1763.87</v>
+      </c>
+      <c r="L18">
+        <v>11.2498</v>
+      </c>
+      <c r="M18">
+        <v>79.59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Remove HotpotQA outputs, update and add datasets
Deleted HotpotQA response CSVs from multiple directories and removed related outputs. Updated datasets/freshqa.csv to fix a date format and removed warning/header lines. Added freshqa_formal.csv and new response/output CSVs for freshqa. Renamed several output files for consistency and moved deprecated hallucination outputs to a test directory. Updated Python scripts and prompt files to reflect these changes.
</commit_message>
<xml_diff>
--- a/stat/data.xlsx
+++ b/stat/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB5BED9-3025-4034-8716-D4AD39290DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5792DB0F-F3E1-4DE2-AA40-E7BB37E5FE77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="15">
   <si>
     <t>gpt-4o</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -80,6 +80,10 @@
   </si>
   <si>
     <t>pass@6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>oa-vs</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -405,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
@@ -468,19 +472,19 @@
         <v>1.5811999999999999</v>
       </c>
       <c r="H3">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="I3">
-        <v>26.53</v>
+        <v>31.08</v>
       </c>
       <c r="J3">
-        <v>3.92</v>
+        <v>3.95</v>
       </c>
       <c r="K3">
-        <v>101.73</v>
+        <v>106.37</v>
       </c>
       <c r="L3">
-        <v>1.4113</v>
+        <v>1.4337</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
@@ -663,19 +667,19 @@
         <v>1.4267000000000001</v>
       </c>
       <c r="H15">
-        <v>16</v>
+        <v>21.33</v>
       </c>
       <c r="I15">
-        <v>69.39</v>
+        <v>62.16</v>
       </c>
       <c r="J15">
-        <v>1.96</v>
+        <v>5.26</v>
       </c>
       <c r="K15">
-        <v>197.15</v>
+        <v>199.29</v>
       </c>
       <c r="L15">
-        <v>1.8134999999999999</v>
+        <v>1.7201</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
@@ -723,22 +727,22 @@
         <v>17.093699999999998</v>
       </c>
       <c r="H18">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="I18">
-        <v>67.349999999999994</v>
+        <v>62.16</v>
       </c>
       <c r="J18">
-        <v>1.96</v>
+        <v>2.63</v>
       </c>
       <c r="K18">
-        <v>1763.87</v>
+        <v>1805.82</v>
       </c>
       <c r="L18">
-        <v>11.2498</v>
+        <v>11.7181</v>
       </c>
       <c r="M18">
-        <v>79.59</v>
+        <v>72.97</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
@@ -759,6 +763,36 @@
       </c>
       <c r="F19">
         <v>240.96270000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>19.329999999999998</v>
+      </c>
+      <c r="I21">
+        <v>65.33</v>
+      </c>
+      <c r="J21">
+        <v>4</v>
+      </c>
+      <c r="K21">
+        <v>596.13</v>
+      </c>
+      <c r="L21">
+        <v>4.4482999999999997</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move and update sample response CSV files
Renamed and relocated several sample response CSV files to the outputs/ directory for consistency. Updated contents of gpt-5_outputs_gpt-5_sample_responses.csv and gpt-5_vs_outputs_gpt-5_sample_responses.csv. Added new presentation slide (slides/20251210.pptx) and updated statistical figures and scripts in the stat/ directory.
</commit_message>
<xml_diff>
--- a/stat/data.xlsx
+++ b/stat/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5792DB0F-F3E1-4DE2-AA40-E7BB37E5FE77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3C6637-286D-433A-9D07-49AEE9F9E2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -547,19 +547,19 @@
         <v>17.4329</v>
       </c>
       <c r="H9">
-        <v>43</v>
+        <v>40.67</v>
       </c>
       <c r="I9">
-        <v>20.41</v>
+        <v>27.03</v>
       </c>
       <c r="J9">
-        <v>7.84</v>
+        <v>9.2100000000000009</v>
       </c>
       <c r="K9">
-        <v>2633.25</v>
+        <v>2293.4899999999998</v>
       </c>
       <c r="L9">
-        <v>30.0015</v>
+        <v>24.464099999999998</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
@@ -610,16 +610,16 @@
         <v>38</v>
       </c>
       <c r="I12">
-        <v>30.61</v>
+        <v>31.08</v>
       </c>
       <c r="J12">
-        <v>7.84</v>
+        <v>7.89</v>
       </c>
       <c r="K12">
-        <v>4222.12</v>
+        <v>3808.19</v>
       </c>
       <c r="L12">
-        <v>42.000700000000002</v>
+        <v>35.700099999999999</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
@@ -701,6 +701,21 @@
       <c r="F16">
         <v>27.958100000000002</v>
       </c>
+      <c r="H16">
+        <v>20</v>
+      </c>
+      <c r="I16">
+        <v>61.33</v>
+      </c>
+      <c r="J16">
+        <v>1.33</v>
+      </c>
+      <c r="K16">
+        <v>188.51</v>
+      </c>
+      <c r="L16">
+        <v>21.434799999999999</v>
+      </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
@@ -793,6 +808,21 @@
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>1</v>
+      </c>
+      <c r="H22">
+        <v>16</v>
+      </c>
+      <c r="I22">
+        <v>68</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>580.04999999999995</v>
+      </c>
+      <c r="L22">
+        <v>36.996099999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add new and update existing data and analysis files
Added new GPT-5 sample response CSVs and updated statistical analysis scripts and figures, including accuracy calculations and data files. These changes support expanded evaluation and updated results for the project.
</commit_message>
<xml_diff>
--- a/stat/data.xlsx
+++ b/stat/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3C6637-286D-433A-9D07-49AEE9F9E2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CAA8110-920F-4A61-BC42-696760BF931F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -506,6 +506,21 @@
       <c r="F4">
         <v>13.4636</v>
       </c>
+      <c r="H4">
+        <v>39.33</v>
+      </c>
+      <c r="I4">
+        <v>24</v>
+      </c>
+      <c r="J4">
+        <v>2.67</v>
+      </c>
+      <c r="K4">
+        <v>87.03</v>
+      </c>
+      <c r="L4">
+        <v>12.4434</v>
+      </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -778,6 +793,24 @@
       </c>
       <c r="F19">
         <v>240.96270000000001</v>
+      </c>
+      <c r="H19">
+        <v>18</v>
+      </c>
+      <c r="I19">
+        <v>64</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>1775.89</v>
+      </c>
+      <c r="L19">
+        <v>187.8108</v>
+      </c>
+      <c r="M19">
+        <v>74.67</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update output paths, add data, and update stats files
Changed output file naming in main.py to use lowercase 'cove' for consistency. Added new sample responses CSV for the search engine. Renamed and moved the gpt-5 CoVe outputs CSV to a new location. Updated statistical analysis scripts, figures, and data files in the 'stat' directory.
</commit_message>
<xml_diff>
--- a/stat/data.xlsx
+++ b/stat/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CAA8110-920F-4A61-BC42-696760BF931F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D03F9188-1F29-484C-8487-87320490562E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -596,6 +596,21 @@
       <c r="F10">
         <v>155.00290000000001</v>
       </c>
+      <c r="H10">
+        <v>32</v>
+      </c>
+      <c r="I10">
+        <v>45.33</v>
+      </c>
+      <c r="J10">
+        <v>9.33</v>
+      </c>
+      <c r="K10">
+        <v>6824.61</v>
+      </c>
+      <c r="L10">
+        <v>202.18029999999999</v>
+      </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" t="s">

</xml_diff>

<commit_message>
Move and update sample responses, update stats and slides
Moved gpt-5 sample responses CSV to outputs/cove-se directory. Updated statistical analysis scripts, figures, and data files in the stat directory. Added new presentation slide for 20251216 and updated 20251210.pptx.
</commit_message>
<xml_diff>
--- a/stat/data.xlsx
+++ b/stat/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A75F67-67A2-4935-9D06-3E0E6C52E28B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4855A375-D10D-46FE-A2E3-DEB4C611DFBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -671,6 +671,21 @@
       <c r="F13">
         <v>78.007099999999994</v>
       </c>
+      <c r="H13">
+        <v>32.67</v>
+      </c>
+      <c r="I13">
+        <v>45.33</v>
+      </c>
+      <c r="J13">
+        <v>10.67</v>
+      </c>
+      <c r="K13">
+        <v>7828.29</v>
+      </c>
+      <c r="L13">
+        <v>142.8083</v>
+      </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" t="s">

</xml_diff>

<commit_message>
Update CSV outputs and statistical analysis scripts
Updated multiple GPT-5 output CSV files with new or revised responses, including file renaming for hotpotqa. Modified stat/calculate.py and stat/calculate2.py, and updated stat/data.xlsx, likely to reflect new data or analysis methods. These changes improve data consistency and support updated statistical evaluation.
</commit_message>
<xml_diff>
--- a/stat/data.xlsx
+++ b/stat/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CB42173-75C0-4087-B277-881D7284AFC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D9F8DAF-9840-4FFE-9600-10488F037FA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -155,17 +155,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -447,12 +443,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD37"/>
+  <dimension ref="A1:X37"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A1" s="4"/>
-      <c r="B1" s="4"/>
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
       <c r="C1" s="2" t="s">
         <v>16</v>
       </c>
@@ -483,585 +479,922 @@
       <c r="V1" s="2"/>
       <c r="W1" s="2"/>
       <c r="X1" s="2"/>
-      <c r="Y1" s="3"/>
-      <c r="Z1" s="3"/>
-      <c r="AA1" s="3"/>
-      <c r="AB1" s="3"/>
-      <c r="AC1" s="3"/>
-      <c r="AD1" s="3"/>
-    </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4" t="s">
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="R2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="V2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="W2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="X2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="2">
         <v>39.81</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="1">
         <v>22.95</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="1">
         <v>49.45</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="1">
         <v>4.7300000000000004</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="1">
         <v>100.61</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="1">
         <v>4.9604999999999997</v>
       </c>
-      <c r="I3" s="4"/>
+      <c r="I3" s="1"/>
       <c r="J3" s="2">
         <v>45.78</v>
       </c>
-      <c r="K3" s="4">
+      <c r="K3" s="1">
         <v>24.6</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="1">
         <v>56.95</v>
       </c>
-      <c r="M3" s="4">
+      <c r="M3" s="1">
         <v>9.0299999999999994</v>
       </c>
-      <c r="N3" s="4"/>
+      <c r="N3" s="1"/>
       <c r="O3" s="2">
         <v>38.03</v>
       </c>
-      <c r="P3" s="4">
+      <c r="P3" s="1">
         <v>28.52</v>
       </c>
-      <c r="Q3" s="4">
+      <c r="Q3" s="1">
         <v>27.16</v>
       </c>
-      <c r="R3" s="4">
+      <c r="R3" s="1">
         <v>1.32</v>
       </c>
-      <c r="S3" s="4"/>
+      <c r="S3" s="1"/>
       <c r="T3" s="2">
         <v>30.33</v>
       </c>
-      <c r="U3" s="4">
+      <c r="U3" s="1">
         <v>11.28</v>
       </c>
-      <c r="V3" s="4">
+      <c r="V3" s="1">
         <v>68.599999999999994</v>
       </c>
-      <c r="W3" s="4">
+      <c r="W3" s="1">
         <v>2.52</v>
       </c>
-      <c r="X3" s="4"/>
-    </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="X3" s="1"/>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="4">
+      <c r="D4" s="1">
         <v>25.03</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="1">
         <v>55.23</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="1">
         <v>12</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="1">
         <v>2253.6799999999998</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="1">
         <v>22.125900000000001</v>
       </c>
-      <c r="I4" s="4"/>
+      <c r="I4" s="1"/>
       <c r="J4" s="2"/>
-      <c r="K4" s="4">
+      <c r="K4" s="1">
         <v>23.38</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="1">
         <v>67.11</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="1">
         <v>15.35</v>
       </c>
-      <c r="N4" s="4"/>
+      <c r="N4" s="1"/>
       <c r="O4" s="2"/>
-      <c r="P4" s="4">
+      <c r="P4" s="1">
         <v>35.9</v>
       </c>
-      <c r="Q4" s="4">
+      <c r="Q4" s="1">
         <v>25.43</v>
       </c>
-      <c r="R4" s="4">
+      <c r="R4" s="1">
         <v>12.17</v>
       </c>
-      <c r="S4" s="4"/>
+      <c r="S4" s="1"/>
       <c r="T4" s="2"/>
-      <c r="U4" s="4">
+      <c r="U4" s="1">
         <v>11.78</v>
       </c>
-      <c r="V4" s="4">
+      <c r="V4" s="1">
         <v>75.209999999999994</v>
       </c>
-      <c r="W4" s="4">
+      <c r="W4" s="1">
         <v>6.12</v>
       </c>
-      <c r="X4" s="4"/>
-    </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="X4" s="1"/>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="4">
+      <c r="D5" s="1">
         <v>25.58</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="1">
         <v>53.72</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="1">
         <v>11.91</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="1">
         <v>3623.59</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="1">
         <v>33.609499999999997</v>
       </c>
-      <c r="I5" s="4"/>
+      <c r="I5" s="1"/>
       <c r="J5" s="2"/>
-      <c r="K5" s="4">
+      <c r="K5" s="1">
         <v>22.4</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="1">
         <v>62.3</v>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="1">
         <v>9.48</v>
       </c>
-      <c r="N5" s="4"/>
+      <c r="N5" s="1"/>
       <c r="O5" s="2"/>
-      <c r="P5" s="4">
+      <c r="P5" s="1">
         <v>38.03</v>
       </c>
-      <c r="Q5" s="4">
+      <c r="Q5" s="1">
         <v>31.47</v>
       </c>
-      <c r="R5" s="4">
+      <c r="R5" s="1">
         <v>19.309999999999999</v>
       </c>
-      <c r="S5" s="4"/>
+      <c r="S5" s="1"/>
       <c r="T5" s="2"/>
-      <c r="U5" s="4">
+      <c r="U5" s="1">
         <v>13.03</v>
       </c>
-      <c r="V5" s="4">
+      <c r="V5" s="1">
         <v>70.25</v>
       </c>
-      <c r="W5" s="4">
+      <c r="W5" s="1">
         <v>5.76</v>
       </c>
-      <c r="X5" s="4"/>
-    </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="X5" s="1"/>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="D6" s="4">
+      <c r="D6" s="1">
         <v>17.579999999999998</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="1">
         <v>65.150000000000006</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="1">
         <v>6.18</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="1">
         <v>207.21</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="1">
         <v>6.4598000000000004</v>
       </c>
-      <c r="I6" s="4"/>
+      <c r="I6" s="1"/>
       <c r="J6" s="2"/>
-      <c r="K6" s="4">
+      <c r="K6" s="1">
         <v>10.4</v>
       </c>
-      <c r="L6" s="4">
+      <c r="L6" s="1">
         <v>85.56</v>
       </c>
-      <c r="M6" s="4">
+      <c r="M6" s="1">
         <v>7</v>
       </c>
-      <c r="N6" s="4"/>
+      <c r="N6" s="1"/>
       <c r="O6" s="2"/>
-      <c r="P6" s="4">
+      <c r="P6" s="1">
         <v>31.97</v>
       </c>
-      <c r="Q6" s="4">
+      <c r="Q6" s="1">
         <v>27.16</v>
       </c>
-      <c r="R6" s="4">
+      <c r="R6" s="1">
         <v>6.88</v>
       </c>
-      <c r="S6" s="4"/>
+      <c r="S6" s="1"/>
       <c r="T6" s="2"/>
-      <c r="U6" s="4">
+      <c r="U6" s="1">
         <v>10.28</v>
       </c>
-      <c r="V6" s="4">
+      <c r="V6" s="1">
         <v>74.38</v>
       </c>
-      <c r="W6" s="4">
+      <c r="W6" s="1">
         <v>3.6</v>
       </c>
-      <c r="X6" s="4"/>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="X6" s="1"/>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="D7" s="4">
+      <c r="D7" s="1">
         <v>15.55</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="1">
         <v>66.709999999999994</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="1">
         <v>3.91</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="1">
         <v>3190.56</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="1">
         <v>17.849</v>
       </c>
       <c r="I7" s="2">
         <v>72.760000000000005</v>
       </c>
       <c r="J7" s="2"/>
-      <c r="K7" s="4">
+      <c r="K7" s="1">
         <v>7.34</v>
       </c>
-      <c r="L7" s="4">
+      <c r="L7" s="1">
         <v>86.9</v>
       </c>
-      <c r="M7" s="4">
+      <c r="M7" s="1">
         <v>2.48</v>
       </c>
       <c r="N7" s="2">
         <v>90.37</v>
       </c>
       <c r="O7" s="2"/>
-      <c r="P7" s="4">
+      <c r="P7" s="1">
         <v>30.49</v>
       </c>
-      <c r="Q7" s="4">
+      <c r="Q7" s="1">
         <v>28.45</v>
       </c>
-      <c r="R7" s="4">
+      <c r="R7" s="1">
         <v>5.29</v>
       </c>
       <c r="S7" s="2">
         <v>39.22</v>
       </c>
       <c r="T7" s="2"/>
-      <c r="U7" s="4">
+      <c r="U7" s="1">
         <v>9.52</v>
       </c>
-      <c r="V7" s="4">
+      <c r="V7" s="1">
         <v>77.69</v>
       </c>
-      <c r="W7" s="4">
+      <c r="W7" s="1">
         <v>4.32</v>
       </c>
       <c r="X7" s="2">
         <v>82.64</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="D8" s="4">
+      <c r="D8" s="1">
         <v>19.11</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="1">
         <v>64.239999999999995</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="1">
         <v>8.1</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="1">
         <v>3441.64</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="1">
         <v>20.038900000000002</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="4">
+      <c r="K8" s="1">
         <v>8.69</v>
       </c>
-      <c r="L8" s="4">
+      <c r="L8" s="1">
         <v>85.56</v>
       </c>
-      <c r="M8" s="4">
+      <c r="M8" s="1">
         <v>3.84</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
-      <c r="P8" s="4">
+      <c r="P8" s="1">
         <v>31.8</v>
       </c>
-      <c r="Q8" s="4">
+      <c r="Q8" s="1">
         <v>29.74</v>
       </c>
-      <c r="R8" s="4">
+      <c r="R8" s="1">
         <v>8.1999999999999993</v>
       </c>
       <c r="S8" s="2"/>
       <c r="T8" s="2"/>
-      <c r="U8" s="4">
+      <c r="U8" s="1">
         <v>21.05</v>
       </c>
-      <c r="V8" s="4">
+      <c r="V8" s="1">
         <v>64.459999999999994</v>
       </c>
-      <c r="W8" s="4">
+      <c r="W8" s="1">
         <v>14.75</v>
       </c>
       <c r="X8" s="2"/>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="2"/>
-      <c r="D9" s="4">
+      <c r="D9" s="1">
         <v>14.07</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="1">
         <v>69.05</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="1">
         <v>2.91</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="1">
         <v>4191.1000000000004</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="1">
         <v>22.114799999999999</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
-      <c r="K9" s="4">
+      <c r="K9" s="1">
         <v>6.61</v>
       </c>
-      <c r="L9" s="4">
+      <c r="L9" s="1">
         <v>87.97</v>
       </c>
-      <c r="M9" s="4">
+      <c r="M9" s="1">
         <v>2.0299999999999998</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
-      <c r="P9" s="4">
+      <c r="P9" s="1">
         <v>26.39</v>
       </c>
-      <c r="Q9" s="4">
+      <c r="Q9" s="1">
         <v>35.78</v>
       </c>
-      <c r="R9" s="4">
+      <c r="R9" s="1">
         <v>3.17</v>
       </c>
       <c r="S9" s="2"/>
       <c r="T9" s="2"/>
-      <c r="U9" s="4">
+      <c r="U9" s="1">
         <v>10.53</v>
       </c>
-      <c r="V9" s="4">
+      <c r="V9" s="1">
         <v>74.38</v>
       </c>
-      <c r="W9" s="4">
+      <c r="W9" s="1">
         <v>3.96</v>
       </c>
       <c r="X9" s="2"/>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="1"/>
-    </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="C10" s="2">
+        <v>19.93</v>
+      </c>
+      <c r="D10" s="1">
+        <v>15.44</v>
+      </c>
+      <c r="E10" s="1">
+        <v>29.4</v>
+      </c>
+      <c r="F10" s="1">
+        <v>1.71</v>
+      </c>
+      <c r="G10" s="1">
+        <v>94.58</v>
+      </c>
+      <c r="H10">
+        <v>12.401999999999999</v>
+      </c>
+      <c r="J10" s="2">
+        <v>25.95</v>
+      </c>
+      <c r="K10" s="1">
+        <v>18.12</v>
+      </c>
+      <c r="L10" s="1">
+        <v>38.68</v>
+      </c>
+      <c r="M10" s="1">
+        <v>2.98</v>
+      </c>
+      <c r="O10" s="2">
+        <v>19.18</v>
+      </c>
+      <c r="P10">
+        <v>17.05</v>
+      </c>
+      <c r="Q10">
+        <v>15.38</v>
+      </c>
+      <c r="R10" s="1">
+        <v>1.01</v>
+      </c>
+      <c r="T10" s="2">
+        <v>8.77</v>
+      </c>
+      <c r="U10">
+        <v>7.52</v>
+      </c>
+      <c r="V10" s="1">
+        <v>20</v>
+      </c>
+      <c r="W10">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="1"/>
-    </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="C11" s="2"/>
+      <c r="D11">
+        <v>17.03</v>
+      </c>
+      <c r="E11">
+        <v>41.76</v>
+      </c>
+      <c r="F11" s="1">
+        <v>6.77</v>
+      </c>
+      <c r="G11">
+        <v>6743.49</v>
+      </c>
+      <c r="H11">
+        <v>114.9687</v>
+      </c>
+      <c r="J11" s="2"/>
+      <c r="K11">
+        <v>16.77</v>
+      </c>
+      <c r="L11" s="1">
+        <v>57.08</v>
+      </c>
+      <c r="M11">
+        <v>7.6</v>
+      </c>
+      <c r="O11" s="2"/>
+      <c r="P11" s="1">
+        <v>22.3</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>17.95</v>
+      </c>
+      <c r="R11" s="1">
+        <v>8.11</v>
+      </c>
+      <c r="T11" s="2"/>
+      <c r="U11" s="1">
+        <v>9.52</v>
+      </c>
+      <c r="V11" s="1">
+        <v>28.57</v>
+      </c>
+      <c r="W11" s="1">
+        <v>3.57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="1"/>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="C12" s="2"/>
+      <c r="D12">
+        <v>15.5</v>
+      </c>
+      <c r="E12">
+        <v>43.68</v>
+      </c>
+      <c r="F12">
+        <v>5.34</v>
+      </c>
+      <c r="G12">
+        <v>7320.52</v>
+      </c>
+      <c r="H12">
+        <v>113.2599</v>
+      </c>
+      <c r="J12" s="2"/>
+      <c r="K12" s="1">
+        <v>13.83</v>
+      </c>
+      <c r="L12">
+        <v>57.55</v>
+      </c>
+      <c r="M12">
+        <v>3.8</v>
+      </c>
+      <c r="O12" s="2"/>
+      <c r="P12">
+        <v>22.62</v>
+      </c>
+      <c r="Q12">
+        <v>15.38</v>
+      </c>
+      <c r="R12" s="1">
+        <v>7.91</v>
+      </c>
+      <c r="T12" s="2"/>
+      <c r="U12">
+        <v>8.02</v>
+      </c>
+      <c r="V12">
+        <v>54.29</v>
+      </c>
+      <c r="W12" s="1">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-    </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="C13" s="2"/>
+      <c r="D13">
+        <v>11.66</v>
+      </c>
+      <c r="E13">
+        <v>49.45</v>
+      </c>
+      <c r="F13">
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="G13">
+        <v>194.27</v>
+      </c>
+      <c r="H13">
+        <v>17.3841</v>
+      </c>
+      <c r="J13" s="2"/>
+      <c r="K13">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="L13">
+        <v>72.17</v>
+      </c>
+      <c r="M13">
+        <v>1.49</v>
+      </c>
+      <c r="O13" s="2"/>
+      <c r="P13">
+        <v>20.16</v>
+      </c>
+      <c r="Q13">
+        <v>10.26</v>
+      </c>
+      <c r="R13">
+        <v>3.65</v>
+      </c>
+      <c r="T13" s="2"/>
+      <c r="U13" s="1">
+        <v>5.76</v>
+      </c>
+      <c r="V13" s="1">
+        <v>42.86</v>
+      </c>
+      <c r="W13" s="1">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="1"/>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="C14" s="2"/>
+      <c r="D14">
+        <v>10.08</v>
+      </c>
+      <c r="E14">
+        <v>51.37</v>
+      </c>
+      <c r="F14">
+        <v>0.48</v>
+      </c>
+      <c r="G14">
+        <v>3227.5</v>
+      </c>
+      <c r="H14">
+        <v>147.7028</v>
+      </c>
+      <c r="I14" s="2">
+        <v>65.11</v>
+      </c>
+      <c r="J14" s="2"/>
+      <c r="K14">
+        <v>7.47</v>
+      </c>
+      <c r="L14">
+        <v>71.23</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2">
+        <v>80.66</v>
+      </c>
+      <c r="O14" s="2"/>
+      <c r="P14">
+        <v>17.05</v>
+      </c>
+      <c r="Q14">
+        <v>16.239999999999998</v>
+      </c>
+      <c r="R14" s="1">
+        <v>1.22</v>
+      </c>
+      <c r="S14" s="2">
+        <v>34.19</v>
+      </c>
+      <c r="T14" s="2"/>
+      <c r="U14">
+        <v>4.76</v>
+      </c>
+      <c r="V14" s="1">
+        <v>48.57</v>
+      </c>
+      <c r="W14" s="1">
+        <v>0.27</v>
+      </c>
+      <c r="X14" s="2">
+        <v>74.290000000000006</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="1"/>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="C15" s="2"/>
+      <c r="D15">
+        <v>9.15</v>
+      </c>
+      <c r="E15">
+        <v>56.59</v>
+      </c>
+      <c r="F15">
+        <v>0.62</v>
+      </c>
+      <c r="G15">
+        <v>3337.4</v>
+      </c>
+      <c r="H15">
+        <v>159.09700000000001</v>
+      </c>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15">
+        <v>5.88</v>
+      </c>
+      <c r="L15">
+        <v>77.36</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15">
+        <v>16.07</v>
+      </c>
+      <c r="Q15">
+        <v>22.22</v>
+      </c>
+      <c r="R15" s="1">
+        <v>1.42</v>
+      </c>
+      <c r="S15" s="2"/>
+      <c r="T15" s="2"/>
+      <c r="U15" s="1">
+        <v>5.26</v>
+      </c>
+      <c r="V15" s="1">
+        <v>45.71</v>
+      </c>
+      <c r="W15" s="1">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="X15" s="2"/>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="1"/>
+      <c r="C16" s="2"/>
+      <c r="D16">
+        <v>7.89</v>
+      </c>
+      <c r="E16">
+        <v>61.54</v>
+      </c>
+      <c r="F16">
+        <v>0.27</v>
+      </c>
+      <c r="G16">
+        <v>3609.91</v>
+      </c>
+      <c r="H16">
+        <v>168.54599999999999</v>
+      </c>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16">
+        <v>5.14</v>
+      </c>
+      <c r="L16">
+        <v>80.19</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
+      <c r="P16">
+        <v>14.1</v>
+      </c>
+      <c r="Q16">
+        <v>29.91</v>
+      </c>
+      <c r="R16" s="1">
+        <v>0.81</v>
+      </c>
+      <c r="S16" s="2"/>
+      <c r="T16" s="2"/>
+      <c r="U16">
+        <v>4.01</v>
+      </c>
+      <c r="V16" s="1">
+        <v>54.29</v>
+      </c>
+      <c r="W16" s="1">
+        <v>0</v>
+      </c>
+      <c r="X16" s="2"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1069,43 +1402,43 @@
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1115,24 +1448,31 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="24">
+    <mergeCell ref="T10:T16"/>
+    <mergeCell ref="N14:N16"/>
+    <mergeCell ref="S14:S16"/>
+    <mergeCell ref="X14:X16"/>
+    <mergeCell ref="J1:N1"/>
+    <mergeCell ref="N7:N9"/>
+    <mergeCell ref="C1:I1"/>
+    <mergeCell ref="C3:C9"/>
+    <mergeCell ref="I14:I16"/>
+    <mergeCell ref="J10:J16"/>
+    <mergeCell ref="X7:X9"/>
+    <mergeCell ref="O1:S1"/>
+    <mergeCell ref="T1:X1"/>
+    <mergeCell ref="O3:O9"/>
+    <mergeCell ref="T3:T9"/>
     <mergeCell ref="A10:A16"/>
     <mergeCell ref="C10:C16"/>
     <mergeCell ref="A17:A23"/>
     <mergeCell ref="A24:A30"/>
     <mergeCell ref="S7:S9"/>
-    <mergeCell ref="X7:X9"/>
-    <mergeCell ref="O1:S1"/>
-    <mergeCell ref="T1:X1"/>
-    <mergeCell ref="O3:O9"/>
-    <mergeCell ref="T3:T9"/>
     <mergeCell ref="A3:A9"/>
     <mergeCell ref="I7:I9"/>
     <mergeCell ref="J3:J9"/>
-    <mergeCell ref="J1:N1"/>
-    <mergeCell ref="N7:N9"/>
-    <mergeCell ref="C1:I1"/>
-    <mergeCell ref="C3:C9"/>
+    <mergeCell ref="O10:O16"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update data sources and Excel file in stat module
Changed CSV file paths in calculate.py and calculate2.py to use new Gemini output files. Updated data.xlsx with new data to reflect these changes.
</commit_message>
<xml_diff>
--- a/stat/data.xlsx
+++ b/stat/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D9F8DAF-9840-4FFE-9600-10488F037FA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D826848F-CCEE-41E5-8083-D0B22505C64F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1354,51 +1354,401 @@
       </c>
       <c r="X16" s="2"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C17" s="2">
+        <v>29.96</v>
+      </c>
+      <c r="D17">
+        <v>23.38</v>
+      </c>
+      <c r="E17">
+        <v>24.5</v>
+      </c>
+      <c r="F17">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="G17">
+        <v>95.45</v>
+      </c>
+      <c r="H17">
+        <v>3.6791999999999998</v>
+      </c>
+      <c r="J17" s="2">
+        <v>28.64</v>
+      </c>
+      <c r="K17">
+        <v>17.38</v>
+      </c>
+      <c r="L17">
+        <v>42.31</v>
+      </c>
+      <c r="M17">
+        <v>1.2</v>
+      </c>
+      <c r="O17" s="2">
+        <v>40.82</v>
+      </c>
+      <c r="P17">
+        <v>38.85</v>
+      </c>
+      <c r="Q17">
+        <v>7.23</v>
+      </c>
+      <c r="R17" s="1">
+        <v>1.66</v>
+      </c>
+      <c r="T17" s="2">
+        <v>16.04</v>
+      </c>
+      <c r="U17">
+        <v>12.03</v>
+      </c>
+      <c r="V17" s="1">
+        <v>26.56</v>
+      </c>
+      <c r="W17" s="1">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C18" s="2"/>
+      <c r="D18">
+        <v>36.31</v>
+      </c>
+      <c r="E18">
+        <v>31.08</v>
+      </c>
+      <c r="F18">
+        <v>22.36</v>
+      </c>
+      <c r="G18">
+        <v>3620.41</v>
+      </c>
+      <c r="H18">
+        <v>26.883299999999998</v>
+      </c>
+      <c r="J18" s="2"/>
+      <c r="K18">
+        <v>31.46</v>
+      </c>
+      <c r="L18">
+        <v>47.86</v>
+      </c>
+      <c r="M18">
+        <v>23.16</v>
+      </c>
+      <c r="O18" s="2"/>
+      <c r="P18">
+        <v>48.2</v>
+      </c>
+      <c r="Q18">
+        <v>14.06</v>
+      </c>
+      <c r="R18" s="1">
+        <v>22.16</v>
+      </c>
+      <c r="T18" s="2"/>
+      <c r="U18">
+        <v>28.07</v>
+      </c>
+      <c r="V18" s="1">
+        <v>35.94</v>
+      </c>
+      <c r="W18" s="1">
+        <v>21.19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
       <c r="B19" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C19" s="2"/>
+      <c r="D19">
+        <v>55.31</v>
+      </c>
+      <c r="E19">
+        <v>14.08</v>
+      </c>
+      <c r="F19">
+        <v>41.14</v>
+      </c>
+      <c r="G19">
+        <v>3227.44</v>
+      </c>
+      <c r="H19">
+        <v>24.215399999999999</v>
+      </c>
+      <c r="J19" s="2"/>
+      <c r="K19">
+        <v>53.12</v>
+      </c>
+      <c r="L19">
+        <v>16.670000000000002</v>
+      </c>
+      <c r="M19">
+        <v>40.82</v>
+      </c>
+      <c r="O19" s="2"/>
+      <c r="P19">
+        <v>66.89</v>
+      </c>
+      <c r="Q19">
+        <v>9.64</v>
+      </c>
+      <c r="R19" s="1">
+        <v>50.69</v>
+      </c>
+      <c r="T19" s="2"/>
+      <c r="U19">
+        <v>42.11</v>
+      </c>
+      <c r="V19">
+        <v>21.88</v>
+      </c>
+      <c r="W19">
+        <v>35.22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C20" s="2"/>
+      <c r="D20">
+        <v>20.87</v>
+      </c>
+      <c r="E20">
+        <v>35.47</v>
+      </c>
+      <c r="F20">
+        <v>2.19</v>
+      </c>
+      <c r="G20">
+        <v>205.87</v>
+      </c>
+      <c r="H20">
+        <v>2.9369000000000001</v>
+      </c>
+      <c r="J20" s="2"/>
+      <c r="K20">
+        <v>14.93</v>
+      </c>
+      <c r="L20">
+        <v>51.71</v>
+      </c>
+      <c r="M20">
+        <v>1.54</v>
+      </c>
+      <c r="O20" s="2"/>
+      <c r="P20">
+        <v>36.72</v>
+      </c>
+      <c r="Q20">
+        <v>17.670000000000002</v>
+      </c>
+      <c r="R20">
+        <v>5.26</v>
+      </c>
+      <c r="T20" s="2"/>
+      <c r="U20">
+        <v>8.77</v>
+      </c>
+      <c r="V20">
+        <v>45.31</v>
+      </c>
+      <c r="W20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
       <c r="B21" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C21" s="2"/>
+      <c r="D21">
+        <v>18.89</v>
+      </c>
+      <c r="E21">
+        <v>39.31</v>
+      </c>
+      <c r="F21">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="G21">
+        <v>3422.22</v>
+      </c>
+      <c r="H21">
+        <v>22.941400000000002</v>
+      </c>
+      <c r="I21" s="2">
+        <v>48.81</v>
+      </c>
+      <c r="J21" s="2"/>
+      <c r="K21">
+        <v>12.48</v>
+      </c>
+      <c r="L21">
+        <v>58.97</v>
+      </c>
+      <c r="M21">
+        <v>1.03</v>
+      </c>
+      <c r="N21" s="2">
+        <v>67.09</v>
+      </c>
+      <c r="O21" s="2"/>
+      <c r="P21">
+        <v>34.590000000000003</v>
+      </c>
+      <c r="Q21">
+        <v>18.07</v>
+      </c>
+      <c r="R21">
+        <v>2.2200000000000002</v>
+      </c>
+      <c r="S21" s="2">
+        <v>30.12</v>
+      </c>
+      <c r="T21" s="2"/>
+      <c r="U21">
+        <v>8.02</v>
+      </c>
+      <c r="V21">
+        <v>50</v>
+      </c>
+      <c r="W21">
+        <v>0</v>
+      </c>
+      <c r="X21" s="2">
+        <v>54.69</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
       <c r="B22" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C22" s="2"/>
+      <c r="D22">
+        <v>17.8</v>
+      </c>
+      <c r="E22">
+        <v>43.33</v>
+      </c>
+      <c r="F22">
+        <v>1.17</v>
+      </c>
+      <c r="G22">
+        <v>3532.35</v>
+      </c>
+      <c r="H22">
+        <v>23.260400000000001</v>
+      </c>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22">
+        <v>10.89</v>
+      </c>
+      <c r="L22">
+        <v>64.959999999999994</v>
+      </c>
+      <c r="M22">
+        <v>1.2</v>
+      </c>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2"/>
+      <c r="P22">
+        <v>33.61</v>
+      </c>
+      <c r="Q22">
+        <v>20.88</v>
+      </c>
+      <c r="R22">
+        <v>2.2200000000000002</v>
+      </c>
+      <c r="S22" s="2"/>
+      <c r="T22" s="2"/>
+      <c r="U22">
+        <v>7.77</v>
+      </c>
+      <c r="V22">
+        <v>51.56</v>
+      </c>
+      <c r="W22">
+        <v>0</v>
+      </c>
+      <c r="X22" s="2"/>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
       <c r="B23" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C23" s="2"/>
+      <c r="D23">
+        <v>16.43</v>
+      </c>
+      <c r="E23">
+        <v>46.62</v>
+      </c>
+      <c r="F23">
+        <v>0.63</v>
+      </c>
+      <c r="G23">
+        <v>4536.21</v>
+      </c>
+      <c r="H23">
+        <v>52.032899999999998</v>
+      </c>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23">
+        <v>10.039999999999999</v>
+      </c>
+      <c r="L23">
+        <v>66.67</v>
+      </c>
+      <c r="M23">
+        <v>0.69</v>
+      </c>
+      <c r="N23" s="2"/>
+      <c r="O23" s="2"/>
+      <c r="P23">
+        <v>30.82</v>
+      </c>
+      <c r="Q23">
+        <v>26.1</v>
+      </c>
+      <c r="R23">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="S23" s="2"/>
+      <c r="T23" s="2"/>
+      <c r="U23">
+        <v>7.52</v>
+      </c>
+      <c r="V23">
+        <v>53.12</v>
+      </c>
+      <c r="W23">
+        <v>0</v>
+      </c>
+      <c r="X23" s="2"/>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -1406,37 +1756,37 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
       <c r="B25" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
       <c r="B26" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
       <c r="B29" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="1" t="s">
         <v>12</v>
@@ -1448,13 +1798,24 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="T10:T16"/>
-    <mergeCell ref="N14:N16"/>
-    <mergeCell ref="S14:S16"/>
-    <mergeCell ref="X14:X16"/>
-    <mergeCell ref="J1:N1"/>
-    <mergeCell ref="N7:N9"/>
+  <mergeCells count="32">
+    <mergeCell ref="T17:T23"/>
+    <mergeCell ref="X21:X23"/>
+    <mergeCell ref="A10:A16"/>
+    <mergeCell ref="C10:C16"/>
+    <mergeCell ref="A17:A23"/>
+    <mergeCell ref="A24:A30"/>
+    <mergeCell ref="S7:S9"/>
+    <mergeCell ref="A3:A9"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="J3:J9"/>
+    <mergeCell ref="O10:O16"/>
+    <mergeCell ref="C17:C23"/>
+    <mergeCell ref="I21:I23"/>
+    <mergeCell ref="J17:J23"/>
+    <mergeCell ref="N21:N23"/>
+    <mergeCell ref="O17:O23"/>
+    <mergeCell ref="S21:S23"/>
     <mergeCell ref="C1:I1"/>
     <mergeCell ref="C3:C9"/>
     <mergeCell ref="I14:I16"/>
@@ -1464,15 +1825,12 @@
     <mergeCell ref="T1:X1"/>
     <mergeCell ref="O3:O9"/>
     <mergeCell ref="T3:T9"/>
-    <mergeCell ref="A10:A16"/>
-    <mergeCell ref="C10:C16"/>
-    <mergeCell ref="A17:A23"/>
-    <mergeCell ref="A24:A30"/>
-    <mergeCell ref="S7:S9"/>
-    <mergeCell ref="A3:A9"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="J3:J9"/>
-    <mergeCell ref="O10:O16"/>
+    <mergeCell ref="T10:T16"/>
+    <mergeCell ref="N14:N16"/>
+    <mergeCell ref="S14:S16"/>
+    <mergeCell ref="X14:X16"/>
+    <mergeCell ref="J1:N1"/>
+    <mergeCell ref="N7:N9"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add sampled datasets, mutation outputs, and repair tools
Add sampled response datasets and mutation test outputs for multiple models, plus repair and sampling utilities. Files added: sampled CSVs for gemini, gpt-5, and qwen3; stability/output CSVs (multiple mutation result files) for each model; repair_with_mutation( _stability / _2 / _3) scripts and tools/random_sample.py for each model directory. Also add a qwen3 sig_responses_fixed dataset. Update stat/data.xlsx and add a temporary Office file (~$data.xlsx). These changes introduce data and scripts to run and analyze mutation-based repair/stability experiments across the three model suites.
</commit_message>
<xml_diff>
--- a/stat/data.xlsx
+++ b/stat/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr-PC\Documents\Workspace\LLMHalluMiti\stat\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zbybr\Documents\Workspace\LLMHalluMiti\stat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF5FB64F-CB79-4499-91A0-B00B58CBBBF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B619EFC8-0885-4134-A1AF-67CCC18C5E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,23 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="62">
   <si>
     <t>gpt-4o</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -152,10 +141,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>overall</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>Method</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
@@ -268,6 +253,22 @@
   </si>
   <si>
     <t>MutRepair</t>
+  </si>
+  <si>
+    <t>RCR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RHR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>OCR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>average</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1131,88 +1132,88 @@
         <v>11</v>
       </c>
       <c r="AA2" s="19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AB2" s="21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AC2" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="AD2" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="AE2" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF2" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="AG2" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="AH2" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="AI2" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="AJ2" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="AK2" s="29" t="s">
+        <v>49</v>
+      </c>
+      <c r="AL2" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="AM2" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="AN2" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="AQ2" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="AR2" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="AS2" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="AT2" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="AW2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AX2" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="AY2" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="AZ2" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="BC2" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="BD2" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="BE2" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="AD2" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="AE2" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF2" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="AG2" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="AH2" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="AI2" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="AJ2" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="AK2" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="AL2" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="AM2" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="AN2" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="AQ2" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="AR2" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="AS2" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="AT2" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="AW2" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="AX2" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="AY2" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="AZ2" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="BC2" s="34" t="s">
-        <v>44</v>
-      </c>
-      <c r="BD2" s="30" t="s">
-        <v>45</v>
-      </c>
-      <c r="BE2" s="35" t="s">
+      <c r="BF2" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="BF2" s="34" t="s">
+      <c r="BG2" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="BG2" s="36" t="s">
-        <v>53</v>
-      </c>
       <c r="BK2" s="39" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="BL2" s="39" t="s">
         <v>17</v>
@@ -1340,13 +1341,13 @@
         <v>24</v>
       </c>
       <c r="BE3" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BF3" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BG3" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="BJ3" s="38" t="s">
         <v>0</v>
@@ -1488,13 +1489,13 @@
         <v>25</v>
       </c>
       <c r="BE4" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BF4" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BG4" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BK4" s="40">
         <v>69.05</v>
@@ -1612,7 +1613,7 @@
       </c>
       <c r="AW5" s="41"/>
       <c r="AX5" s="24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="AY5" s="25">
         <v>3623.59</v>
@@ -1622,16 +1623,16 @@
       </c>
       <c r="BC5" s="42"/>
       <c r="BD5" s="23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="BE5" s="33" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BF5" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BG5" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BK5" s="40">
         <f>BK4-BK3</f>
@@ -1753,7 +1754,7 @@
       </c>
       <c r="AW6" s="42"/>
       <c r="AX6" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AY6" s="27">
         <v>2095.5500000000002</v>
@@ -1768,13 +1769,13 @@
         <v>24</v>
       </c>
       <c r="BE6" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BF6" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BG6" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BK6" s="40">
         <f>BK5/BK3*100</f>
@@ -1858,7 +1859,7 @@
       </c>
       <c r="AA7" s="42"/>
       <c r="AB7" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AC7" s="50"/>
       <c r="AD7" s="14">
@@ -1907,13 +1908,13 @@
         <v>25</v>
       </c>
       <c r="BE7" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BF7" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BG7" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BJ7" s="38" t="s">
         <v>1</v>
@@ -2040,16 +2041,16 @@
       </c>
       <c r="BC8" s="42"/>
       <c r="BD8" s="23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="BE8" s="33" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BF8" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BG8" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BK8" s="40">
         <v>61.54</v>
@@ -2155,7 +2156,7 @@
       </c>
       <c r="AW9" s="41"/>
       <c r="AX9" s="24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="AY9" s="25">
         <v>7320.52</v>
@@ -2170,10 +2171,10 @@
         <v>24</v>
       </c>
       <c r="BE9" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BF9" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BG9" s="6">
         <v>0.157</v>
@@ -2292,7 +2293,7 @@
       </c>
       <c r="AW10" s="42"/>
       <c r="AX10" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AY10" s="27">
         <v>1804.96</v>
@@ -2305,13 +2306,13 @@
         <v>25</v>
       </c>
       <c r="BE10" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BF10" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BG10" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BK10" s="40">
         <f>BK9/BK7*100</f>
@@ -2383,7 +2384,7 @@
       </c>
       <c r="AA11" s="42"/>
       <c r="AB11" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AC11" s="50"/>
       <c r="AD11" s="14">
@@ -2429,16 +2430,16 @@
       </c>
       <c r="BC11" s="42"/>
       <c r="BD11" s="23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="BE11" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BF11" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BG11" s="37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="BJ11" s="38" t="s">
         <v>13</v>
@@ -2566,13 +2567,13 @@
         <v>24</v>
       </c>
       <c r="BE12" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="BF12" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="BG12" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="BK12" s="40">
         <v>46.62</v>
@@ -2674,7 +2675,7 @@
       </c>
       <c r="AW13" s="41"/>
       <c r="AX13" s="24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="AY13" s="25">
         <v>3227.44</v>
@@ -2687,13 +2688,13 @@
         <v>25</v>
       </c>
       <c r="BE13" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="BF13" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="BG13" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="BK13" s="40">
         <f>BK12-BK11</f>
@@ -2811,7 +2812,7 @@
       </c>
       <c r="AW14" s="42"/>
       <c r="AX14" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AY14" s="27">
         <v>2268.11</v>
@@ -2821,16 +2822,16 @@
       </c>
       <c r="BC14" s="42"/>
       <c r="BD14" s="23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="BE14" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="BF14" s="37" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="BG14" s="37" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="BK14" s="40">
         <f>BK13/BK11*100</f>
@@ -2906,7 +2907,7 @@
       <c r="X15" s="44"/>
       <c r="AA15" s="42"/>
       <c r="AB15" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AC15" s="50"/>
       <c r="AD15" s="14">
@@ -3183,7 +3184,7 @@
       </c>
       <c r="AW17" s="41"/>
       <c r="AX17" s="24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="AY17" s="25">
         <v>3219.47</v>
@@ -3295,7 +3296,7 @@
       </c>
       <c r="AW18" s="42"/>
       <c r="AX18" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AY18" s="27">
         <v>2260.54</v>
@@ -3373,7 +3374,7 @@
       </c>
       <c r="AA19" s="42"/>
       <c r="AB19" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="AC19" s="50"/>
       <c r="AD19" s="14">
@@ -4031,18 +4032,18 @@
     <row r="34" spans="2:23" ht="15" x14ac:dyDescent="0.2">
       <c r="B34" s="2"/>
       <c r="C34" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="E34" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="35" spans="2:23" x14ac:dyDescent="0.2">
       <c r="B35" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C35" s="2">
         <v>15</v>
@@ -4056,7 +4057,7 @@
     </row>
     <row r="36" spans="2:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B36" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C36" s="2">
         <v>17.22</v>
@@ -4068,18 +4069,18 @@
         <v>4.95</v>
       </c>
       <c r="U36" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="V36" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="V36" s="19" t="s">
+      <c r="W36" s="20" t="s">
         <v>48</v>
-      </c>
-      <c r="W36" s="20" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="37" spans="2:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B37" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C37" s="2">
         <v>17.22</v>
@@ -4091,7 +4092,7 @@
         <v>2.97</v>
       </c>
       <c r="U37" s="45" t="s">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="V37" s="45"/>
       <c r="W37" s="46"/>
@@ -4132,13 +4133,13 @@
     <row r="41" spans="2:23" ht="15" x14ac:dyDescent="0.2">
       <c r="B41" s="22"/>
       <c r="C41" s="12" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="U41" s="14">
         <v>14.07</v>

</xml_diff>